<commit_message>
Add Streamlit course, DBMS chapter images, and refresh MCQ banks
- New standalone Streamlit course (content/Streamlit/): 8 reading-material
  lessons plus README, following a single running placement-tool scenario
- Add illustrations for DBMS Unit 1 Ch4 (Relational Algebra), Unit 2 Ch1
  (ER Modeling), and Unit 2 Ch2 (Normalization), with matching image
  references added to each lesson
- Refresh Units 1-6 MCQ banks and Unit 4 output exports

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="Rbeaf4f365a8d4e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="Rac999c01ea394013"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,7 +281,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="74" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
@@ -292,10 +292,10 @@
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="36" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="36" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="36" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="38" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="38" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="38" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -352,13 +352,13 @@
         <x:v>answer</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A2" s="5" t="str">
         <x:v>Python - MCQ - 4.1.1</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
         <x:v>A school attendance system has a list of roll numbers for today's class. It must mark attendance once for each roll number already present in the list.
-Which loop is the best fit for this requirement?</x:v>
+Which loop should the system use to process each roll number cleanly?</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
         <x:v>A for loop is best when the program already has a sequence of items to visit. Here, the roll-number list decides exactly what must be processed, so Python can take one roll number at a time without a manually managed counter.</x:v>
@@ -404,13 +404,13 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="3" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A3" s="5" t="str">
         <x:v>Python - MCQ - 4.1.2</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
         <x:v>A cafe billing app keeps accepting item names until the cashier types `done`.
-Which loop condition best matches this sentinel-based requirement?</x:v>
+The cashier has not fixed the number of items in advance. Which loop condition should the billing app use to keep accepting items until the stop word appears?</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
         <x:v>A sentinel loop repeats until a special value appears. The loop should continue while the item is not `done` and stop as soon as `done` is entered.</x:v>
@@ -456,13 +456,13 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="4" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A4" s="5" t="str">
         <x:v>Python - MCQ - 4.1.3</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
         <x:v>A quiz app must display question numbers 1, 2, 3, 4, and 5 before starting a round.
-Which line should replace the blank?
+Which line should replace the blank so the app shows exactly those five question numbers?
 ```python
 for q_no in ______:
     print(q_no)
@@ -512,13 +512,13 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="5" t="str">
         <x:v>Python - MCQ - 4.1.4</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>A contact app must show each contact with a serial number like `1. Asha`, `2. Ravi`, and `3. Mina`.
-Which concept makes this cleanest?</x:v>
+        <x:v>A contact app must show each contact with a serial number, such as `1. Asha`, `2. Ravi`, and `3. Mina`.
+Which loop technique should the app use so each contact is shown with the correct serial number?</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>`enumerate()` gives both the index/position and the item during each loop pass. With `start=1`, the numbering matches the user-facing serial numbers.</x:v>
@@ -564,12 +564,12 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="6" ht="132" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="str">
         <x:v>Python - MCQ - 4.1.5</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>An order system skips unavailable items.
+        <x:v>An order system skips items that are marked as unavailable.
 ```python
 items = ["tea", "sold out", "coffee"]
 for item in items:
@@ -577,7 +577,7 @@
         continue
     print(item)
 ```
-What is printed?</x:v>
+A customer views the available-item list. Which items will the system show to the customer?</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
         <x:v>`continue` skips only the current iteration. The sold-out item is skipped, but the loop continues and prints tea and coffee.</x:v>
@@ -623,12 +623,12 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="7" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A7" s="5" t="str">
         <x:v>Python - MCQ - 4.1.6</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>A scholarship checker stops when it finds the first score of 90 or above.
+        <x:v>A scholarship checker scans scores in order and should stop as soon as it finds the first score of 90 or above.
 ```python
 scores = [72, 88, 91, 95]
 for score in scores:
@@ -636,7 +636,7 @@
         print(score)
         break
 ```
-What is printed?</x:v>
+Which score will the checker display as the first qualifying score?</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
         <x:v>The loop checks scores in order. 72 and 88 do not qualify. 91 qualifies, so it is printed and `break` stops the loop before 95 is checked.</x:v>
@@ -682,12 +682,12 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="8" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A8" s="5" t="str">
         <x:v>Python - MCQ - 4.1.7</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>A search program reports when an item is missing.
+        <x:v>A search program checks a stationery box for an eraser.
 ```python
 target = "eraser"
 for item in ["pen", "pencil", "scale"]:
@@ -697,7 +697,7 @@
 else:
     print("Missing")
 ```
-What is printed?</x:v>
+The box does not contain an eraser. What message will the search program show?</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
         <x:v>The target is never found, so `break` never runs. A loop's `else` block runs only when the loop finishes without a break, so it prints Missing.</x:v>
@@ -743,19 +743,19 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="9" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A9" s="5" t="str">
         <x:v>Python - MCQ - 4.1.8</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>A pattern-printing program creates a small triangle.
+        <x:v>A pattern-printing tool creates a small triangle for a terminal display.
 ```python
 for row in range(1, 4):
     for col in range(row):
         print("*", end="")
     print()
 ```
-What is printed?</x:v>
+When the display is generated, which star pattern will appear on the screen?</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>The outer loop uses row values 1, 2, and 3. The inner loop prints that many stars on each row, and the final `print()` moves to the next line.</x:v>
@@ -807,18 +807,18 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="10" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A10" s="5" t="str">
         <x:v>Python - MCQ - 4.1.9</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>A retry loop currently gives four attempts by mistake.
+        <x:v>A retry screen should allow exactly three attempts, but the current loop allows one extra attempt.
 ```python
 attempts = 0
 while attempts &lt;= 3:
     attempts += 1
 ```
-What change gives exactly three attempts?</x:v>
+Which change should the developer make so the retry screen allows exactly three attempts?</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
         <x:v>Starting from 0, the condition `attempts &lt; 3` runs for attempts 0, 1, and 2. The original `&lt;= 3` runs one extra time.</x:v>
@@ -864,13 +864,13 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A11" s="5" t="str">
         <x:v>Python - MCQ - 4.1.10</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>A weather app must find the highest temperature in a list that may contain only negative values.
-Which initialization is safest?</x:v>
+        <x:v>A weather app must find the highest temperature in a list, and some cities may have only negative temperatures.
+Which initialization lets the app still find the correct highest temperature for a list like `[-5, -2, -9]`?</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
         <x:v>Starting with the first actual list value avoids assuming that the maximum is non-negative. Initializing to 0 would fail for all-negative lists.</x:v>
@@ -916,7 +916,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="12" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
         <x:v>Python - MCQ - 4.2.1</x:v>
       </x:c>
@@ -927,7 +927,7 @@
 for ch in code:
     print(ch)
 ```
-What is printed?</x:v>
+When the badge code is revealed character by character, what will the printer output?</x:v>
       </x:c>
       <x:c r="C12" s="5" t="str">
         <x:v>Strings are sequences, so the loop visits each character in order: A, then I, then 2. Each print call uses a new line by default.</x:v>
@@ -973,7 +973,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="13" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
         <x:v>Python - MCQ - 4.2.2</x:v>
       </x:c>
@@ -985,7 +985,7 @@
     print(count)
     count += 1
 ```
-Why does this code fail before it can print anything?</x:v>
+Before the ticket counter can run, what problem will Python report?</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
         <x:v>The `while` statement must end with a colon. Because the colon after `count &lt;= 3` is missing, Python raises a syntax error before running the loop body.</x:v>
@@ -1031,7 +1031,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
         <x:v>Python - MCQ - 4.2.3</x:v>
       </x:c>
@@ -1043,7 +1043,7 @@
     print("Try", attempt)
     attempt += 1
 ```
-How many times does the loop body run?</x:v>
+How many attempt messages will the retry screen show?</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
         <x:v>The loop runs for attempt values 1, 2, and 3. After the third run, attempt becomes 4, making `attempt &lt;= 3` false.</x:v>
@@ -1089,7 +1089,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
         <x:v>Python - MCQ - 4.2.4</x:v>
       </x:c>
@@ -1099,7 +1099,7 @@
 for slot in range(5, 5):
     print(slot)
 ```
-What happens?</x:v>
+When the scheduler runs, what slot numbers will it show?</x:v>
       </x:c>
       <x:c r="C15" s="5" t="str">
         <x:v>`range(5, 5)` is empty because the start and stop are the same, and the stop value is excluded. The loop body never runs.</x:v>
@@ -1145,7 +1145,7 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="16" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
         <x:v>Python - MCQ - 4.2.5</x:v>
       </x:c>
@@ -1156,7 +1156,7 @@
 while seconds &gt; 0:
     print(seconds)
 ```
-Which line should be added inside the loop to make it stop correctly?</x:v>
+Which line should be added inside the loop so the countdown shows 3, 2, 1 and then stops?</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
         <x:v>The loop condition depends on `seconds`, so `seconds` must move toward 0 on every pass. Subtracting 1 after printing gives 3, 2, 1 and then stops.</x:v>
@@ -1202,7 +1202,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="17" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
         <x:v>Python - MCQ - 4.2.6</x:v>
       </x:c>
@@ -1212,7 +1212,7 @@
 for n in range(0, 10, 2):
     print(n)
 ```
-The requirement changes: print even numbers from 10 down to 2. Which range should be used?</x:v>
+The requirement changes: the display should show even numbers from 10 down to 2. Which `range()` call should the display use?</x:v>
       </x:c>
       <x:c r="C17" s="5" t="str">
         <x:v>For a countdown, the step must be negative. `range(10, 1, -2)` produces 10, 8, 6, 4, 2 because it stops before 1.</x:v>
@@ -1258,19 +1258,19 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="18" ht="132" hidden="0" customHeight="1">
       <x:c r="A18" s="5" t="str">
         <x:v>Python - MCQ - 4.2.7</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>A developer wrote this repeated code.
+        <x:v>A developer wrote this repeated backup message by copying the same line four times.
 ```python
 print("Backup started")
 print("Backup started")
 print("Backup started")
 print("Backup started")
 ```
-Which replacement is cleanest if the message must be printed exactly four times?</x:v>
+Which replacement should the developer use so the backup tool shows the same message exactly four times with cleaner code?</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
         <x:v>A for loop with `range(4)` expresses four repetitions directly and avoids copying the same print statement multiple times.</x:v>
@@ -1316,7 +1316,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="19" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A19" s="5" t="str">
         <x:v>Python - MCQ - 4.2.8</x:v>
       </x:c>
@@ -1328,7 +1328,7 @@
     print(checkpoint)
     checkpoint += 1
 ```
-What is printed?</x:v>
+When the progress indicator runs, which checkpoint numbers will appear?</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
         <x:v>The loop runs for checkpoint values 0, 1, 2, and 3. When checkpoint becomes 4, the condition `checkpoint &lt; 4` becomes false.</x:v>
@@ -1374,17 +1374,17 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="20" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A20" s="5" t="str">
         <x:v>Python - MCQ - 4.2.9</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
-        <x:v>A login script is written as follows.
+        <x:v>A login script checks the entered PIN before asking the user for input.
 ```python
 while pin != "1234":
     pin = input("PIN: ")
 ```
-Why can this code fail before asking for input?</x:v>
+Why can this login script fail before the first PIN prompt appears?</x:v>
       </x:c>
       <x:c r="C20" s="5" t="str">
         <x:v>The condition checks `pin` before any value has been assigned to it. `pin` should be initialized before the while loop, such as `pin = ""`.</x:v>
@@ -1436,7 +1436,7 @@
       </x:c>
       <x:c r="B21" s="5" t="str">
         <x:v>A security app should allow at most 3 wrong password attempts.
-Which version correctly moves the loop toward stopping?</x:v>
+Which version correctly updates the attempt count so the security app can stop after the third wrong attempt?</x:v>
       </x:c>
       <x:c r="C21" s="5" t="str">
         <x:v>The safe version initializes attempts, checks the limit, and increments attempts inside the loop. Without the increment, the loop may never reach the stopping condition.</x:v>
@@ -1491,7 +1491,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="22" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A22" s="5" t="str">
         <x:v>Python - MCQ - 4.2.11</x:v>
       </x:c>
@@ -1503,7 +1503,7 @@
 while stock &gt; 0:
     stock = stock - packed
 ```
-What is the risk in this code?</x:v>
+When this stock-checking loop runs, what problem can occur?</x:v>
       </x:c>
       <x:c r="C22" s="5" t="str">
         <x:v>Since `packed` is 0, `stock` never changes from 10. The condition remains true forever, causing an infinite loop.</x:v>
@@ -1549,7 +1549,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="132" hidden="0" customHeight="1">
+    <x:row r="23" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A23" s="5" t="str">
         <x:v>Python - MCQ - 4.2.12</x:v>
       </x:c>
@@ -1563,7 +1563,7 @@
     total += scores[i]
     i += 1
 ```
-What is the final value of `total`?</x:v>
+After all survey scores are processed, what total will the system store?</x:v>
       </x:c>
       <x:c r="C23" s="5" t="str">
         <x:v>The loop adds scores[0], scores[1], and scores[2]: 4 + 0 + 5. The final total is 9.</x:v>
@@ -1609,13 +1609,13 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="24" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A24" s="5" t="str">
         <x:v>Python - MCQ - 4.2.13</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
-        <x:v>A form should keep asking for age until the value is between 18 and 60, inclusive.
-Which condition should be used in the while loop?</x:v>
+        <x:v>A registration form should keep asking for age until the value is between 18 and 60, inclusive.
+Which loop condition should the form use while the entered age is still invalid?</x:v>
       </x:c>
       <x:c r="C24" s="5" t="str">
         <x:v>The loop should continue while the age is invalid. Ages below 18 or above 60 are invalid, so `age &lt; 18 or age &gt; 60` is the correct condition.</x:v>
@@ -1661,13 +1661,13 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="25" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A25" s="5" t="str">
         <x:v>Python - MCQ - 4.2.14</x:v>
       </x:c>
       <x:c r="B25" s="5" t="str">
         <x:v>A chatbot keeps reading messages until the user types `bye`. The number of messages is not known beforehand.
-Which loop pattern is being used?</x:v>
+Which loop pattern is the chatbot using to decide when the conversation should stop?</x:v>
       </x:c>
       <x:c r="C25" s="5" t="str">
         <x:v>This is a sentinel-controlled loop. It stops when a special signal value, `bye`, appears rather than after a fixed count.</x:v>
@@ -1713,7 +1713,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="26" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A26" s="5" t="str">
         <x:v>Python - MCQ - 4.2.15</x:v>
       </x:c>
@@ -1725,7 +1725,7 @@
     print(n)
     n += 1
 ```
-Is the claim correct?</x:v>
+When the ticket display runs, is the developer's claim correct?</x:v>
       </x:c>
       <x:c r="C26" s="5" t="str">
         <x:v>The condition is `n &lt; 5`, so the loop prints 1, 2, 3, and 4 only. To include 5, the condition would need to be `n &lt;= 5`.</x:v>
@@ -1771,7 +1771,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="27" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A27" s="5" t="str">
         <x:v>Python - MCQ - 4.2.16</x:v>
       </x:c>
@@ -1781,7 +1781,7 @@
 for q in range(1, 6):
     print(q)
 ```
-Why does the app stop at 5 instead of printing 6?</x:v>
+The app shows 1 through 5, but not 6. Why does the question-number display stop before 6?</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str">
         <x:v>`range(start, stop)` includes the start value but excludes the stop value. Therefore, `range(1, 6)` produces 1 through 5.</x:v>
@@ -1827,7 +1827,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="28" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A28" s="5" t="str">
         <x:v>Python - MCQ - 4.2.17</x:v>
       </x:c>
@@ -1837,7 +1837,7 @@
 for n in range(10, 0, -3):
     print(n, end=" ")
 ```
-What is printed?</x:v>
+When the countdown display runs, which numbers will appear?</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
         <x:v>The range starts at 10 and subtracts 3 each time while staying above 0. It produces 10, 7, 4, and 1.</x:v>
@@ -1883,18 +1883,18 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="29" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A29" s="5" t="str">
         <x:v>Python - MCQ - 4.2.18</x:v>
       </x:c>
       <x:c r="B29" s="5" t="str">
-        <x:v>A developer wants to print each product name, but writes:
+        <x:v>A developer wants to show each product name, but writes:
 ```python
 products = ["pen", "bag", "book"]
 for i in products:
     print(products[i])
 ```
-Why is this wrong?</x:v>
+When the product display runs, why will this code fail?</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str">
         <x:v>In `for i in products`, `i` becomes each product string, such as `"pen"`, not a numeric index. Using a string as a list index causes an error.</x:v>
@@ -1940,18 +1940,18 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="30" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A30" s="5" t="str">
         <x:v>Python - MCQ - 4.2.19</x:v>
       </x:c>
       <x:c r="B30" s="5" t="str">
         <x:v>A leaderboard should display ranks starting from 1.
-Which line should replace the blank?
 ```python
 players = ["Asha", "Ravi"]
 for rank, player in ______:
     print(rank, player)
-```</x:v>
+```
+Which line should replace the blank so the leaderboard shows each player with the correct rank?</x:v>
       </x:c>
       <x:c r="C30" s="5" t="str">
         <x:v>`enumerate(players, start=1)` produces pairs `(1, "Asha")` and `(2, "Ravi")`, giving both the rank and the player.</x:v>
@@ -1997,17 +1997,17 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="31" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A31" s="5" t="str">
         <x:v>Python - MCQ - 4.2.20</x:v>
       </x:c>
       <x:c r="B31" s="5" t="str">
-        <x:v>A developer writes:
+        <x:v>A developer writes this loop to display names:
 ```python
 for i in range(len(names)):
     print(names[i])
 ```
-If the index is not needed, which replacement is cleaner?</x:v>
+If the app only needs each name and does not need the index, which replacement is cleaner?</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
         <x:v>When only the item is needed, direct iteration is clearer and avoids unnecessary index handling.</x:v>
@@ -2057,24 +2057,24 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="132" hidden="0" customHeight="1">
+    <x:row r="32" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A32" s="5" t="str">
         <x:v>Python - MCQ - 4.2.21</x:v>
       </x:c>
       <x:c r="B32" s="5" t="str">
-        <x:v>A data-cleaning loop should keep only positive numbers.
+        <x:v>A data-cleaning loop should add only positive numbers to a running total.
 ```python
 values = [3, -1, 4]
-clean = []
+total = 0
 for v in values:
     if v &lt; 0:
         continue
-    clean.append(v)
-```
-What is the final value of `clean`?</x:v>
+    total = total + v
+```
+After the loop finishes, what total will the program store?</x:v>
       </x:c>
       <x:c r="C32" s="5" t="str">
-        <x:v>When v is -1, `continue` skips the append. The positive values 3 and 4 are appended, so clean becomes `[3, 4]`.</x:v>
+        <x:v>The loop adds 3, skips -1 because `continue` jumps to the next iteration, and then adds 4. The final total is 7.</x:v>
       </x:c>
       <x:c r="D32" s="5" t="n">
         <x:v>1</x:v>
@@ -2102,22 +2102,22 @@
       </x:c>
       <x:c r="L32" s="5"/>
       <x:c r="M32" s="5" t="str">
-        <x:v>[3, -1, 4]</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N32" s="5" t="str">
-        <x:v>[-1]</x:v>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="O32" s="5" t="str">
-        <x:v>[3, 4]</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="P32" s="5" t="str">
-        <x:v>[]</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Q32" s="5" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="132" hidden="0" customHeight="1">
+    <x:row r="33" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A33" s="5" t="str">
         <x:v>Python - MCQ - 4.2.22</x:v>
       </x:c>
@@ -2131,7 +2131,7 @@
         valid = False
         break
 ```
-Does this code meet the requirement?</x:v>
+Does this validator correctly reject the batch when it reaches the first negative quantity?</x:v>
       </x:c>
       <x:c r="C33" s="5" t="str">
         <x:v>Yes. The loop checks quantities one by one, sets `valid` to False at the first negative value, and uses `break` to stop checking the rest.</x:v>
@@ -2177,13 +2177,13 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="34" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A34" s="5" t="str">
         <x:v>Python - MCQ - 4.2.23</x:v>
       </x:c>
       <x:c r="B34" s="5" t="str">
         <x:v>A seating chart checks 3 rows, and each row has 4 seats.
-If the outer loop runs 3 times and the inner loop runs 4 times for each outer pass, how many seat checks happen?</x:v>
+If the outer loop checks each row and the inner loop checks each seat in that row, how many seat checks will the seating-chart system perform?</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str">
         <x:v>Nested loop work multiplies: 3 outer passes x 4 inner passes = 12 total checks.</x:v>
@@ -2229,12 +2229,12 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="171.60000610351562" hidden="0" customHeight="1">
+    <x:row r="35" ht="184.8000030517578" hidden="0" customHeight="1">
       <x:c r="A35" s="5" t="str">
         <x:v>Python - MCQ - 4.2.24</x:v>
       </x:c>
       <x:c r="B35" s="5" t="str">
-        <x:v>A developer wants this output:
+        <x:v>A developer wants this two-row pattern on a terminal screen:
 ```text
 ***
 ***
@@ -2246,7 +2246,7 @@
         print("*", end="")
 print()
 ```
-What is wrong?</x:v>
+When the terminal pattern is generated, why will the rows not appear correctly?</x:v>
       </x:c>
       <x:c r="C35" s="5" t="str">
         <x:v>The newline `print()` is outside the outer loop, so it runs only once after all stars are printed. It should be indented inside the outer loop, after the inner loop.</x:v>
@@ -2292,7 +2292,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="36" ht="132" hidden="0" customHeight="1">
       <x:c r="A36" s="5" t="str">
         <x:v>Python - MCQ - 4.2.25</x:v>
       </x:c>
@@ -2305,7 +2305,7 @@
     if amount &gt; 0:
         total += amount
 ```
-What is the final value of `total`?</x:v>
+After the donation list is processed, what total will the app store?</x:v>
       </x:c>
       <x:c r="C36" s="5" t="str">
         <x:v>Only positive amounts are added. The loop adds 100 and 50, while -20 and 0 are ignored, so the total is 150.</x:v>
@@ -2351,13 +2351,13 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="37" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A37" s="5" t="str">
         <x:v>Python - MCQ - 4.2.26</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>A multiplication-table app should print rows for 1, 2, and 3 and columns for 1, 2, and 3.
-Which nested loop header pair is correct?</x:v>
+        <x:v>A multiplication-table app should generate rows for 1, 2, and 3 and columns for 1, 2, and 3.
+Which nested-loop header pair should the app use to generate the 3 by 3 table?</x:v>
       </x:c>
       <x:c r="C37" s="5" t="str">
         <x:v>`range(1, 4)` produces 1, 2, and 3. Using it for both row and column creates the required 3 by 3 table.</x:v>
@@ -2407,12 +2407,12 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="38" ht="132" hidden="0" customHeight="1">
       <x:c r="A38" s="5" t="str">
         <x:v>Python - MCQ - 4.2.27</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>A program finds the largest number like this:
+        <x:v>A program tries to find the largest number in an empty list.
 ```python
 numbers = []
 largest = numbers[0]
@@ -2420,7 +2420,7 @@
     if n &gt; largest:
         largest = n
 ```
-What happens for the empty list?</x:v>
+When the program starts processing this empty list, what will happen?</x:v>
       </x:c>
       <x:c r="C38" s="5" t="str">
         <x:v>The code tries to access `numbers[0]`, but an empty list has no first element. Python raises an IndexError before the loop starts.</x:v>
@@ -2466,13 +2466,13 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="39" ht="66" hidden="0" customHeight="1">
       <x:c r="A39" s="5" t="str">
         <x:v>Python - MCQ - 4.2.28</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
-        <x:v>A comparison tool checks every user against every course using nested loops. There are 100 users and 100 courses.
-How many comparisons are made?</x:v>
+        <x:v>A course recommendation tool compares every user against every course. There are 100 users and 100 courses.
+If the tool uses one loop for users and a nested loop for courses, how many comparisons will it perform?</x:v>
       </x:c>
       <x:c r="C39" s="5" t="str">
         <x:v>The inner loop runs 100 times for each of the 100 users, so the total is 100 x 100 = 10,000 comparisons.</x:v>
@@ -2518,19 +2518,19 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="40" ht="132" hidden="0" customHeight="1">
       <x:c r="A40" s="5" t="str">
         <x:v>Python - MCQ - 4.2.29</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
-        <x:v>A pattern currently grows by row.
+        <x:v>A terminal pattern currently grows by row.
 ```python
 for row in range(1, 4):
     for col in range(row):
         print("#", end="")
     print()
 ```
-The new requirement is to print exactly 3 hashes on every row for 3 rows. What should change?</x:v>
+The new requirement is to show exactly 3 hashes on every row for 3 rows. What should the developer change?</x:v>
       </x:c>
       <x:c r="C40" s="5" t="str">
         <x:v>The current inner range depends on `row`, so the width changes. Using `range(3)` for the inner loop prints exactly three hashes on every row.</x:v>
@@ -2576,7 +2576,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="132" hidden="0" customHeight="1">
+    <x:row r="41" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A41" s="5" t="str">
         <x:v>Python - MCQ - 4.2.30</x:v>
       </x:c>
@@ -2590,7 +2590,7 @@
         all_positive = False
         break
 ```
-What is the final value of `all_positive`, and why?</x:v>
+After the payment checker reaches the zero amount, what final value will it store in `all_positive`?</x:v>
       </x:c>
       <x:c r="C41" s="5" t="str">
         <x:v>The loop reaches amount 0, which is not positive. It sets `all_positive` to False and breaks, so the final value is False.</x:v>
@@ -2639,7 +2639,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2e7e97434d41ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8318f5c331c426e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix MCQ consistency in units 4 and 5
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="R1dfa595974a04008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="R4d3313ba56aa42bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,12 +30,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -49,7 +59,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -75,6 +85,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -391,55 +407,55 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
-      <x:c r="A1" s="8" t="str">
+      <x:c r="A1" s="11" t="str">
         <x:v>title</x:v>
       </x:c>
-      <x:c r="B1" s="8" t="str">
+      <x:c r="B1" s="11" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="C1" s="8" t="str">
+      <x:c r="C1" s="11" t="str">
         <x:v>explanation</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="str">
+      <x:c r="D1" s="11" t="str">
         <x:v>score</x:v>
       </x:c>
-      <x:c r="E1" s="8" t="str">
+      <x:c r="E1" s="11" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="F1" s="11" t="str">
         <x:v>difficulty</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="str">
+      <x:c r="G1" s="11" t="str">
         <x:v>bloomTaxonomy</x:v>
       </x:c>
-      <x:c r="H1" s="8" t="str">
+      <x:c r="H1" s="11" t="str">
         <x:v>tags</x:v>
       </x:c>
-      <x:c r="I1" s="8" t="str">
+      <x:c r="I1" s="11" t="str">
         <x:v>subjects</x:v>
       </x:c>
-      <x:c r="J1" s="8" t="str">
+      <x:c r="J1" s="11" t="str">
         <x:v>topics</x:v>
       </x:c>
-      <x:c r="K1" s="8" t="str">
+      <x:c r="K1" s="11" t="str">
         <x:v>subTopics</x:v>
       </x:c>
-      <x:c r="L1" s="8" t="str">
+      <x:c r="L1" s="11" t="str">
         <x:v>companies</x:v>
       </x:c>
-      <x:c r="M1" s="8" t="str">
+      <x:c r="M1" s="11" t="str">
         <x:v>option1</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="11" t="str">
         <x:v>option2</x:v>
       </x:c>
-      <x:c r="O1" s="8" t="str">
+      <x:c r="O1" s="11" t="str">
         <x:v>option3</x:v>
       </x:c>
-      <x:c r="P1" s="8" t="str">
+      <x:c r="P1" s="11" t="str">
         <x:v>option4</x:v>
       </x:c>
-      <x:c r="Q1" s="8" t="str">
+      <x:c r="Q1" s="11" t="str">
         <x:v>answer</x:v>
       </x:c>
     </x:row>
@@ -452,7 +468,7 @@
 Which loop should the scanner use to visit every ID cleanly?</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>A for loop is best when the program already has a sequence of items to visit. Here, the roll-number list decides exactly what must be processed, so Python can take one roll number at a time without a manually managed counter.</x:v>
+        <x:v>A `for` loop is best when the program already has a sequence of package IDs to visit. Python can take one ID at a time without a manually managed counter.</x:v>
       </x:c>
       <x:c r="D2" s="9" t="n">
         <x:v>1</x:v>
@@ -480,16 +496,16 @@
       </x:c>
       <x:c r="L2" s="9"/>
       <x:c r="M2" s="9" t="str">
-        <x:v>A recursive function, because attendance needs repetition</x:v>
+        <x:v>A recursive function that repeatedly rescans the package-ID list until an external stop condition is met</x:v>
       </x:c>
       <x:c r="N2" s="9" t="str">
-        <x:v>An if statement for each possible roll number</x:v>
+        <x:v>A separate `if` statement for every possible package ID</x:v>
       </x:c>
       <x:c r="O2" s="9" t="str">
         <x:v>A while loop that runs forever and stops manually</x:v>
       </x:c>
       <x:c r="P2" s="9" t="str">
-        <x:v>A for loop that iterates through the roll-number list</x:v>
+        <x:v>A `for` loop that iterates through the package-ID list</x:v>
       </x:c>
       <x:c r="Q2" s="9" t="n">
         <x:v>4</x:v>
@@ -719,18 +735,18 @@
         <x:v>Python - MCQ - 4.1.6</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>A scholarship checker scans scores in order and should stop as soon as it finds the first score of 90 or above.
-```python
-scores = [72, 88, 91, 95]
-for score in scores:
-    if score &gt;= 90:
-        print(score)
+        <x:v>A quality monitor scans sensor readings in order and should stop as soon as it finds the first reading of 90 or above.
+```python
+readings = [72, 88, 91, 95]
+for reading in readings:
+    if reading &gt;= 90:
+        print(reading)
         break
 ```
-Which score will the checker display as the first qualifying score?</x:v>
+Which reading will the monitor identify as the first threshold breach?</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>The loop checks scores in order. 72 and 88 do not qualify. 91 qualifies, so it is printed and `break` stops the loop before 95 is checked.</x:v>
+        <x:v>The loop checks readings in order. 72 and 88 are below the threshold. 91 qualifies, so it is reported and `break` stops the loop before 95 is checked.</x:v>
       </x:c>
       <x:c r="D7" s="9" t="n">
         <x:v>1</x:v>
@@ -2569,7 +2585,7 @@
 If the service uses one loop for customers and a nested loop for products, how many comparisons will it perform?</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
-        <x:v>The inner loop runs 100 times for each of the 100 users, so the total is 100 x 100 = 10,000 comparisons.</x:v>
+        <x:v>The inner loop runs 100 times for each of the 100 customers, so the total is 100 × 100 = 10,000 product comparisons.</x:v>
       </x:c>
       <x:c r="D39" s="9" t="n">
         <x:v>1</x:v>
@@ -2733,7 +2749,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b859afc40aa42b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64431399a67e4bb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>